<commit_message>
Add attachment consolidation and harden automation workflows
</commit_message>
<xml_diff>
--- a/config/outlook/OAS-K_Outlook-Revisi_Configuration.xlsx
+++ b/config/outlook/OAS-K_Outlook-Revisi_Configuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Project\OfficeAutomationSuite-Karina\config\outlook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354D0BE9-81AB-43AA-9C62-A3556FA4EABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F28391-CFA5-4F04-A75D-20DBDF0CD301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -425,18 +425,6 @@
     <t>VALIDATION_FAILED</t>
   </si>
   <si>
-    <t>Dear {SENDER_NAME},
-Status penarikan data Attendance untuk payroll {PERIOD}:
-GAGAL
-Data revisi belum dapat diproses karena:
-{ERROR_REASON}
-Silakan perbaiki dan kirim ulang paling lambat:
-{RESUBMIT_DEADLINE}
-Terima Kasih
-Best Regards,
-This message is generated automatically by Karina Robot.</t>
-  </si>
-  <si>
     <t>SUMMARY_PIC</t>
   </si>
   <si>
@@ -462,6 +450,20 @@
   </si>
   <si>
     <t>Placeholder utama: {SENDER_NAME}, {PERIOD}, {ORIGINAL_SUBJECT}, {REQUIRED_CC_EMAIL}, {RESUBMIT_DEADLINE}, {ERROR_REASON}, {TOTAL_EMAIL}, {SUCCESS_EMAIL}, {FAILED_EMAIL}, {OUTPUT_TXT_COUNT}, {OUTPUT_FOLDER}</t>
+  </si>
+  <si>
+    <t>Dear {SENDER_NAME},
+Status penarikan data Attendance untuk payroll {PERIOD}:
+GAGAL
+Data revisi belum dapat diproses karena:
+{ERROR_REASON}
+Silakan perbaiki dan kirim ulang paling lambat:
+{RESUBMIT_DEADLINE}
+Pastikan Subject email adalah sbb :
+{EXPECTED_SUBJECT}
+Terima Kasih
+Best Regards,
+This message is generated automatically by Karina Robot.</t>
   </si>
 </sst>
 </file>
@@ -782,6 +784,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -791,9 +796,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -971,18 +973,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
@@ -1201,7 +1203,7 @@
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="B24" s="36"/>
+      <c r="B24" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1239,26 +1241,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:7" ht="22.65" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
@@ -1749,30 +1751,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
     </row>
     <row r="2" spans="1:9" ht="22.65" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="28" t="s">
@@ -4556,18 +4558,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
@@ -4700,18 +4702,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
@@ -4845,20 +4847,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:4" ht="22.65" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
@@ -5117,24 +5119,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" spans="1:6" ht="22.65" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
@@ -5213,7 +5215,7 @@
         <v>120</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="100" customHeight="1">
@@ -5221,19 +5223,19 @@
         <v>9</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -5253,14 +5255,14 @@
       <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" ht="29.4" customHeight="1">
-      <c r="A11" s="35" t="s">
-        <v>133</v>
-      </c>
-      <c r="B11" s="33"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
+      <c r="A11" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4"/>

</xml_diff>